<commit_message>
Changes on sebastian folder
</commit_message>
<xml_diff>
--- a/Sebastian Nduva - USIU - 265res - 2026/distribution_descriptive_statistics.xlsx
+++ b/Sebastian Nduva - USIU - 265res - 2026/distribution_descriptive_statistics.xlsx
@@ -459,13 +459,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.709</v>
+        <v>3.766</v>
       </c>
       <c r="C2" t="n">
-        <v>1.268</v>
+        <v>0.278</v>
       </c>
       <c r="D2" t="n">
-        <v>1.126</v>
+        <v>0.528</v>
       </c>
     </row>
     <row r="3">
@@ -475,13 +475,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3.683</v>
+        <v>3.792</v>
       </c>
       <c r="C3" t="n">
-        <v>1.323</v>
+        <v>0.271</v>
       </c>
       <c r="D3" t="n">
-        <v>1.15</v>
+        <v>0.521</v>
       </c>
     </row>
     <row r="4">
@@ -491,13 +491,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.721</v>
+        <v>3.789</v>
       </c>
       <c r="C4" t="n">
-        <v>1.164</v>
+        <v>0.311</v>
       </c>
       <c r="D4" t="n">
-        <v>1.079</v>
+        <v>0.5580000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -507,13 +507,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.706</v>
+        <v>3.792</v>
       </c>
       <c r="C5" t="n">
-        <v>1.224</v>
+        <v>0.271</v>
       </c>
       <c r="D5" t="n">
-        <v>1.106</v>
+        <v>0.521</v>
       </c>
     </row>
     <row r="6">
@@ -523,13 +523,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.717</v>
+        <v>3.819</v>
       </c>
       <c r="C6" t="n">
-        <v>1.166</v>
+        <v>0.278</v>
       </c>
       <c r="D6" t="n">
-        <v>1.08</v>
+        <v>0.527</v>
       </c>
     </row>
   </sheetData>
@@ -575,13 +575,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.709</v>
+        <v>3.766</v>
       </c>
       <c r="C2" t="n">
-        <v>1.268</v>
+        <v>0.278</v>
       </c>
       <c r="D2" t="n">
-        <v>1.126</v>
+        <v>0.528</v>
       </c>
     </row>
     <row r="3">
@@ -591,13 +591,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3.683</v>
+        <v>3.792</v>
       </c>
       <c r="C3" t="n">
-        <v>1.323</v>
+        <v>0.271</v>
       </c>
       <c r="D3" t="n">
-        <v>1.15</v>
+        <v>0.521</v>
       </c>
     </row>
     <row r="4">
@@ -607,13 +607,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.721</v>
+        <v>3.789</v>
       </c>
       <c r="C4" t="n">
-        <v>1.164</v>
+        <v>0.311</v>
       </c>
       <c r="D4" t="n">
-        <v>1.079</v>
+        <v>0.5580000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -623,13 +623,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.706</v>
+        <v>3.792</v>
       </c>
       <c r="C5" t="n">
-        <v>1.224</v>
+        <v>0.271</v>
       </c>
       <c r="D5" t="n">
-        <v>1.106</v>
+        <v>0.521</v>
       </c>
     </row>
     <row r="6">
@@ -639,13 +639,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.717</v>
+        <v>3.819</v>
       </c>
       <c r="C6" t="n">
-        <v>1.166</v>
+        <v>0.278</v>
       </c>
       <c r="D6" t="n">
-        <v>1.08</v>
+        <v>0.527</v>
       </c>
     </row>
   </sheetData>
@@ -691,13 +691,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.709</v>
+        <v>3.766</v>
       </c>
       <c r="C2" t="n">
-        <v>1.268</v>
+        <v>0.278</v>
       </c>
       <c r="D2" t="n">
-        <v>1.126</v>
+        <v>0.528</v>
       </c>
     </row>
     <row r="3">
@@ -707,13 +707,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3.683</v>
+        <v>3.792</v>
       </c>
       <c r="C3" t="n">
-        <v>1.323</v>
+        <v>0.271</v>
       </c>
       <c r="D3" t="n">
-        <v>1.15</v>
+        <v>0.521</v>
       </c>
     </row>
     <row r="4">
@@ -723,13 +723,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.721</v>
+        <v>3.789</v>
       </c>
       <c r="C4" t="n">
-        <v>1.164</v>
+        <v>0.311</v>
       </c>
       <c r="D4" t="n">
-        <v>1.079</v>
+        <v>0.5580000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -739,13 +739,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3.706</v>
+        <v>3.792</v>
       </c>
       <c r="C5" t="n">
-        <v>1.224</v>
+        <v>0.271</v>
       </c>
       <c r="D5" t="n">
-        <v>1.106</v>
+        <v>0.521</v>
       </c>
     </row>
     <row r="6">
@@ -755,13 +755,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.717</v>
+        <v>3.819</v>
       </c>
       <c r="C6" t="n">
-        <v>1.166</v>
+        <v>0.278</v>
       </c>
       <c r="D6" t="n">
-        <v>1.08</v>
+        <v>0.527</v>
       </c>
     </row>
   </sheetData>

</xml_diff>